<commit_message>
- update | update `MachineListPage`, `TestProposalPage`, `TicketManagementPage` to handle many category of machine (add new/edit machine, excel import) - add | add category filter in `MachineListPage`, `LocationTrackPage`
</commit_message>
<xml_diff>
--- a/frontend/public/Mau_Excel_MayMoc.xlsx
+++ b/frontend/public/Mau_Excel_MayMoc.xlsx
@@ -1,14 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\react\tpm\frontend\public\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2435EA43-0994-40D3-8E78-2118619C6F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF86C157-133C-4E44-A894-A394E86E1F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,24 +12,14 @@
     <sheet name="LoaiMayMoc" sheetId="2" r:id="rId2"/>
     <sheet name="HangSX" sheetId="3" r:id="rId3"/>
     <sheet name="NhaCungCap" sheetId="4" r:id="rId4"/>
+    <sheet name="PhanLoai" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
   <si>
     <t>Serial</t>
   </si>
@@ -42,15 +27,39 @@
     <t>Loại máy</t>
   </si>
   <si>
+    <t>Đặc tính</t>
+  </si>
+  <si>
+    <t>Phân loại</t>
+  </si>
+  <si>
     <t>Model máy</t>
   </si>
   <si>
     <t>Hãng sản xuất</t>
   </si>
   <si>
+    <t>Nhà cung cấp</t>
+  </si>
+  <si>
     <t>RFID</t>
   </si>
   <si>
+    <t>NFC</t>
+  </si>
+  <si>
+    <t>Công suất (W)</t>
+  </si>
+  <si>
+    <t>Áp suất (MPa)</t>
+  </si>
+  <si>
+    <t>Điện áp (V)</t>
+  </si>
+  <si>
+    <t>Lưu lượng khí nén (lít/phút)</t>
+  </si>
+  <si>
     <t>Giá (VNĐ)</t>
   </si>
   <si>
@@ -69,12 +78,27 @@
     <t>SERIAL-MAU-001</t>
   </si>
   <si>
+    <t>Bàn hút</t>
+  </si>
+  <si>
+    <t>10x20</t>
+  </si>
+  <si>
     <t>Model-XYZ-123</t>
   </si>
   <si>
+    <t>BAOYU</t>
+  </si>
+  <si>
+    <t>GIANG THÀNH</t>
+  </si>
+  <si>
     <t>RFID-12345</t>
   </si>
   <si>
+    <t>NFC-12345</t>
+  </si>
+  <si>
     <t>15/01/2023</t>
   </si>
   <si>
@@ -84,81 +108,51 @@
     <t>SERIAL-MAU-002</t>
   </si>
   <si>
+    <t>Bộ điều tiết thun</t>
+  </si>
+  <si>
+    <t>20x30</t>
+  </si>
+  <si>
     <t>Model-PK-456</t>
   </si>
   <si>
     <t>RFID-67890</t>
   </si>
   <si>
+    <t>NFC-67890</t>
+  </si>
+  <si>
     <t>20/02/2024</t>
   </si>
   <si>
     <t>Ghi chú cho phụ kiện mẫu 2</t>
   </si>
   <si>
-    <t>NFC</t>
-  </si>
-  <si>
-    <t>NFC-12345</t>
-  </si>
-  <si>
-    <t>NFC-67890</t>
-  </si>
-  <si>
-    <t>Bàn hút</t>
-  </si>
-  <si>
-    <t>Bộ điều tiết thun</t>
-  </si>
-  <si>
-    <t>BAOYU</t>
-  </si>
-  <si>
-    <t>Nhà cung cấp</t>
-  </si>
-  <si>
-    <t>Đặc tính</t>
-  </si>
-  <si>
-    <t>10x20</t>
-  </si>
-  <si>
-    <t>20x30</t>
-  </si>
-  <si>
-    <t>GIANG THÀNH</t>
-  </si>
-  <si>
-    <t>Công suất (W)</t>
-  </si>
-  <si>
-    <t>Áp suất (MPa)</t>
-  </si>
-  <si>
-    <t>Điện áp (V)</t>
-  </si>
-  <si>
-    <t>Lưu lượng khí nén (lít/phút)</t>
+    <t>Máy móc thiết bị</t>
+  </si>
+  <si>
+    <t>Phụ tùng vật tư</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -168,8 +162,10 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -209,26 +205,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -562,215 +556,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="28" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" hidden="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" customWidth="1"/>
+    <col min="10" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="26.7109375" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="28" customWidth="1"/>
+    <col min="16" max="16" width="14.140625" customWidth="1"/>
+    <col min="17" max="17" width="22.140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="27" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="20" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
       <c r="F1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2">
-        <v>10</v>
-      </c>
-      <c r="J2">
+      <c r="K2">
         <v>15</v>
-      </c>
-      <c r="K2">
-        <v>20</v>
       </c>
       <c r="L2">
         <v>20</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2">
+        <v>20</v>
+      </c>
+      <c r="N2" s="1">
         <v>150000000</v>
       </c>
-      <c r="N2" t="s">
-        <v>13</v>
-      </c>
-      <c r="O2">
+      <c r="O2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2">
         <v>10</v>
       </c>
-      <c r="P2" s="3">
+      <c r="Q2" s="1">
         <v>150000000</v>
       </c>
-      <c r="Q2" t="s">
-        <v>14</v>
+      <c r="R2" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M3" s="3">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N3" s="1">
         <v>5000000</v>
       </c>
-      <c r="N3" t="s">
-        <v>18</v>
-      </c>
-      <c r="O3">
+      <c r="O3" t="s">
+        <v>34</v>
+      </c>
+      <c r="P3">
         <v>5</v>
       </c>
-      <c r="P3" s="3">
+      <c r="Q3" s="1">
         <v>5000000</v>
       </c>
-      <c r="Q3" t="s">
-        <v>19</v>
+      <c r="R3" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="M1:Q1 M2:O3 Q2:Q3 A2:A3 D2:D3 G1:G3 D1:E1 A1:B1" numberStoredAsText="1"/>
-  </ignoredErrors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A235E470-EFC7-49E0-B06E-31C3A85CD3FF}">
-          <x14:formula1>
-            <xm:f>LoaiMayMoc!$A:$A</xm:f>
-          </x14:formula1>
-          <xm:sqref>B2:B1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CBE0319C-AC79-4F98-98FE-959DA43B7DF1}">
-          <x14:formula1>
-            <xm:f>HangSX!$A:$A</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2:E1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{61D70CBA-93CC-45AF-85D1-5A24C6AC0E32}">
-          <x14:formula1>
-            <xm:f>NhaCungCap!$A:$A</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2:F1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{472E5E5B-407E-4F2E-BAC6-82849E509BD9}">
-          <x14:formula1>
-            <xm:f>LoaiMayMoc!$B:$B</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C1048576</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{983E5464-CEE9-41EE-8EED-83216360782C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -779,7 +751,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04243702-2A7A-45A5-BBE3-5C41301554E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -788,7 +760,16 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{078887F3-BA3E-484B-B931-5F112A68A033}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>